<commit_message>
fixing tests in frontend. Complete open API contract has endpoints on side of backend
</commit_message>
<xml_diff>
--- a/test_trip_export.xlsx
+++ b/test_trip_export.xlsx
@@ -1,18 +1,18 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet name="Přehled" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet name="Denní plány" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet name="Recepty" sheetId="3" state="visible" r:id="rId3"/>
-    <sheet name="Nákupní seznam" sheetId="4" state="visible" r:id="rId4"/>
-    <sheet name="Nutriční analýza" sheetId="5" state="visible" r:id="rId5"/>
-    <sheet name="Náklady" sheetId="6" state="visible" r:id="rId6"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Přehled" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Denní plány" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Recepty" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Nákupní seznam" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Nutriční analýza" sheetId="5" state="visible" r:id="rId5"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Náklady" sheetId="6" state="visible" r:id="rId6"/>
   </sheets>
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Denní plány'!$A$3:$G$8</definedName>
@@ -244,13 +244,13 @@
 </file>
 
 <file path=xl/charts/chart1.xml><?xml version="1.0" encoding="utf-8"?>
-<chartSpace xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns="http://schemas.openxmlformats.org/drawingml/2006/chart">
+<chartSpace xmlns="http://schemas.openxmlformats.org/drawingml/2006/chart">
   <chart>
     <title>
       <tx>
         <rich>
-          <a:bodyPr/>
-          <a:p>
+          <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
+          <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
             <a:pPr>
               <a:defRPr/>
             </a:pPr>
@@ -273,7 +273,7 @@
             </strRef>
           </tx>
           <spPr>
-            <a:ln>
+            <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
               <a:prstDash val="solid"/>
             </a:ln>
           </spPr>
@@ -301,13 +301,13 @@
 </file>
 
 <file path=xl/charts/chart2.xml><?xml version="1.0" encoding="utf-8"?>
-<chartSpace xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns="http://schemas.openxmlformats.org/drawingml/2006/chart">
+<chartSpace xmlns="http://schemas.openxmlformats.org/drawingml/2006/chart">
   <chart>
     <title>
       <tx>
         <rich>
-          <a:bodyPr/>
-          <a:p>
+          <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
+          <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
             <a:pPr>
               <a:defRPr/>
             </a:pPr>
@@ -330,14 +330,14 @@
             </strRef>
           </tx>
           <spPr>
-            <a:ln>
+            <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
               <a:prstDash val="solid"/>
             </a:ln>
           </spPr>
           <marker>
             <symbol val="none"/>
             <spPr>
-              <a:ln>
+              <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
                 <a:prstDash val="solid"/>
               </a:ln>
             </spPr>
@@ -365,8 +365,8 @@
         <title>
           <tx>
             <rich>
-              <a:bodyPr/>
-              <a:p>
+              <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
+              <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
                 <a:pPr>
                   <a:defRPr/>
                 </a:pPr>
@@ -392,8 +392,8 @@
         <title>
           <tx>
             <rich>
-              <a:bodyPr/>
-              <a:p>
+              <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
+              <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
                 <a:pPr>
                   <a:defRPr/>
                 </a:pPr>
@@ -419,7 +419,7 @@
 </file>
 
 <file path=xl/drawings/drawing1.xml><?xml version="1.0" encoding="utf-8"?>
-<wsDr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing">
+<wsDr xmlns="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing">
   <oneCellAnchor>
     <from>
       <col>3</col>
@@ -434,9 +434,9 @@
         <cNvGraphicFramePr/>
       </nvGraphicFramePr>
       <xfrm/>
-      <a:graphic>
+      <a:graphic xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
         <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
-          <c:chart r:id="rId1"/>
+          <c:chart xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1"/>
         </a:graphicData>
       </a:graphic>
     </graphicFrame>
@@ -456,9 +456,9 @@
         <cNvGraphicFramePr/>
       </nvGraphicFramePr>
       <xfrm/>
-      <a:graphic>
+      <a:graphic xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
         <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
-          <c:chart r:id="rId2"/>
+          <c:chart xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId2"/>
         </a:graphicData>
       </a:graphic>
     </graphicFrame>
@@ -783,7 +783,7 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>11.07.2025</t>
+          <t>12.07.2025</t>
         </is>
       </c>
     </row>
@@ -795,7 +795,7 @@
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>15.07.2025</t>
+          <t>16.07.2025</t>
         </is>
       </c>
     </row>
@@ -1078,7 +1078,7 @@
       </c>
       <c r="B4" s="6" t="inlineStr">
         <is>
-          <t>11.07.2025</t>
+          <t>12.07.2025</t>
         </is>
       </c>
       <c r="C4" s="8" t="inlineStr">
@@ -1107,7 +1107,7 @@
       </c>
       <c r="B5" s="6" t="inlineStr">
         <is>
-          <t>11.07.2025</t>
+          <t>12.07.2025</t>
         </is>
       </c>
       <c r="C5" s="9" t="inlineStr">
@@ -1136,7 +1136,7 @@
       </c>
       <c r="B6" s="6" t="inlineStr">
         <is>
-          <t>11.07.2025</t>
+          <t>12.07.2025</t>
         </is>
       </c>
       <c r="C6" s="10" t="inlineStr">
@@ -1165,7 +1165,7 @@
       </c>
       <c r="B7" s="6" t="inlineStr">
         <is>
-          <t>12.07.2025</t>
+          <t>13.07.2025</t>
         </is>
       </c>
       <c r="C7" s="8" t="inlineStr">
@@ -1194,7 +1194,7 @@
       </c>
       <c r="B8" s="6" t="inlineStr">
         <is>
-          <t>12.07.2025</t>
+          <t>13.07.2025</t>
         </is>
       </c>
       <c r="C8" s="9" t="inlineStr">

</xml_diff>